<commit_message>
Fix issues regarding last commits
</commit_message>
<xml_diff>
--- a/config/Configuration-Test.xlsx
+++ b/config/Configuration-Test.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -64,37 +64,37 @@
     <t xml:space="preserve">StartHour</t>
   </si>
   <si>
+    <t xml:space="preserve">MISSION00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single-Agent Test (Multi-Camera)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENVIRONMENT00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROUP02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-150.0, 150.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(30.0, 150.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PX4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(13/12/2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(16:30:00)</t>
+  </si>
+  <si>
     <t xml:space="preserve">X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Single-Agent Test (Multi-Camera)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENVIRONMENT00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAM00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(-150.0, 150.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(30.0, 150.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PX4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(13/12/2024)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(16:30:00)</t>
   </si>
   <si>
     <t xml:space="preserve">MISSION01</t>
@@ -869,10 +869,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -944,8 +945,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
+      <b val="true"/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1041,7 +1043,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1094,6 +1096,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1118,10 +1124,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1131,6 +1133,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1614,13 +1620,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="21" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="21" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="54.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="2" width="26.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="29.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="29.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="30.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="2" width="20.92"/>
@@ -1679,38 +1685,36 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="8"/>
+      <c r="B3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="G3" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="H3" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="I3" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="J3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="K3" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
@@ -1759,7 +1763,9 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8"/>
+      <c r="A4" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="B4" s="9" t="s">
         <v>22</v>
       </c>
@@ -1767,28 +1773,28 @@
         <v>23</v>
       </c>
       <c r="D4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>14</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>15</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>24</v>
       </c>
       <c r="G4" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="I4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="J4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="K4" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L4" s="12"/>
       <c r="M4" s="12"/>
@@ -1845,28 +1851,28 @@
         <v>26</v>
       </c>
       <c r="D5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="9" t="s">
         <v>14</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>15</v>
       </c>
       <c r="F5" s="11" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="I5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="J5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="K5" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L5" s="12"/>
       <c r="M5" s="12"/>
@@ -1923,28 +1929,28 @@
         <v>29</v>
       </c>
       <c r="D6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>14</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>15</v>
       </c>
       <c r="F6" s="11" t="s">
         <v>30</v>
       </c>
       <c r="G6" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="I6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="J6" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="9" t="s">
+      <c r="K6" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L6" s="12"/>
       <c r="M6" s="12"/>
@@ -2028,7 +2034,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD16"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="2" width="29.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="40.25"/>
@@ -2100,21 +2106,21 @@
       <c r="B3" s="22" t="s">
         <v>274</v>
       </c>
-      <c r="C3" s="22" t="b">
+      <c r="C3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D3" s="22" t="s">
         <v>275</v>
       </c>
-      <c r="E3" s="22" t="b">
+      <c r="E3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="F3" s="22" t="s">
         <v>276</v>
       </c>
-      <c r="G3" s="22" t="b">
+      <c r="G3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2167,7 +2173,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="33.54"/>
@@ -2180,12 +2186,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -2207,7 +2213,7 @@
     </row>
     <row r="3" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>33</v>
@@ -2215,7 +2221,7 @@
       <c r="C3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="15" t="s">
         <v>35</v>
       </c>
     </row>
@@ -2229,7 +2235,7 @@
       <c r="C4" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="15" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2258,7 +2264,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:BM1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="38.38"/>
@@ -2269,15 +2275,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -2373,7 +2379,7 @@
       <c r="D3" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E3" s="15" t="n">
+      <c r="E3" s="16" t="n">
         <v>2</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -2454,7 +2460,7 @@
       <c r="D4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="16" t="n">
         <v>4</v>
       </c>
       <c r="F4" s="9" t="s">
@@ -2530,12 +2536,12 @@
         <v>54</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="16" t="n">
         <v>8</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -2616,7 +2622,7 @@
       <c r="D6" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="16" t="n">
         <v>16</v>
       </c>
       <c r="F6" s="9" t="s">
@@ -2710,7 +2716,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -2720,7 +2726,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="29.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="36.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="2" width="26.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="29.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="29.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="26.66"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16" min="12" style="12" width="11"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16379" min="17" style="2" width="11"/>
@@ -2729,50 +2735,50 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
       <c r="XFC1" s="3"/>
       <c r="XFD1" s="3"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="18" t="s">
         <v>67</v>
       </c>
       <c r="L2" s="12"/>
@@ -2787,260 +2793,260 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="18" t="s">
+      <c r="C3" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="18" t="n">
+      <c r="H3" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I3" s="18" t="n">
+      <c r="I3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="18" t="n">
+      <c r="J3" s="19" t="n">
         <v>12000</v>
       </c>
       <c r="XFC3" s="3"/>
       <c r="XFD3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="H4" s="18" t="n">
+      <c r="H4" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="18" t="n">
+      <c r="I4" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="18" t="n">
+      <c r="J4" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="I5" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="J5" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="H6" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="I6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="H7" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I7" s="18" t="n">
+      <c r="I7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="18" t="n">
+      <c r="J7" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I8" s="18" t="n">
+      <c r="I8" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="18" t="n">
+      <c r="J8" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H9" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I9" s="18" t="n">
+      <c r="I9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J9" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="H10" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I10" s="18" t="n">
+      <c r="I10" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="18" t="n">
+      <c r="J10" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -3077,7 +3083,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD23"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -3093,32 +3099,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>94</v>
       </c>
       <c r="H2" s="12"/>
@@ -3134,22 +3140,22 @@
       <c r="XFD2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="18" t="n">
+      <c r="D3" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G3" s="2"/>
@@ -3159,22 +3165,22 @@
       <c r="XEY3" s="3"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="D4" s="18" t="n">
+      <c r="D4" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G4" s="2"/>
@@ -3184,22 +3190,22 @@
       <c r="XEY4" s="3"/>
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="D5" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G5" s="2"/>
@@ -3209,22 +3215,22 @@
       <c r="XEY5" s="3"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="D6" s="18" t="n">
+      <c r="D6" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G6" s="2"/>
@@ -3234,22 +3240,22 @@
       <c r="XEY6" s="3"/>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G7" s="2"/>
@@ -3259,22 +3265,22 @@
       <c r="XEY7" s="3"/>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G8" s="2"/>
@@ -3284,22 +3290,22 @@
       <c r="XEY8" s="3"/>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G9" s="2"/>
@@ -3309,22 +3315,22 @@
       <c r="XEY9" s="3"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G10" s="2"/>
@@ -3369,7 +3375,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.28"/>
@@ -3383,53 +3389,53 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
       <c r="L1" s="2"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="18" t="s">
         <v>116</v>
       </c>
       <c r="M2" s="12"/>
@@ -3437,878 +3443,868 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I3" s="18" t="n">
+      <c r="I3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="18" t="n">
+      <c r="J3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="18" t="n">
+      <c r="K3" s="19" t="n">
         <v>3</v>
       </c>
       <c r="L3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="H4" s="18" t="s">
+      <c r="H4" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="I4" s="18" t="n">
+      <c r="I4" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J4" s="18" t="n">
+      <c r="J4" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="18" t="n">
+      <c r="K4" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="I5" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="J5" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K5" s="18" t="n">
+      <c r="K5" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="H6" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="I6" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="H7" s="18" t="s">
+      <c r="H7" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="I7" s="18" t="n">
+      <c r="I7" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J7" s="18" t="n">
+      <c r="J7" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K7" s="18" t="n">
+      <c r="K7" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L7" s="2"/>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="H8" s="18" t="s">
+      <c r="H8" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I8" s="18" t="n">
+      <c r="I8" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="18" t="n">
+      <c r="J8" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K8" s="18" t="n">
+      <c r="K8" s="19" t="n">
         <v>3</v>
       </c>
       <c r="L8" s="2"/>
       <c r="XFD8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>145</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="H9" s="18" t="s">
+      <c r="H9" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I9" s="18" t="n">
+      <c r="I9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K9" s="18" t="n">
+      <c r="K9" s="19" t="n">
         <v>3</v>
       </c>
       <c r="L9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="H10" s="18" t="s">
+      <c r="H10" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="I10" s="18" t="n">
+      <c r="I10" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J10" s="18" t="n">
+      <c r="J10" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K10" s="18" t="n">
+      <c r="K10" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>149</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G11" s="18" t="s">
+      <c r="G11" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="H11" s="18" t="s">
+      <c r="H11" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I11" s="18" t="n">
+      <c r="I11" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J11" s="18" t="n">
+      <c r="J11" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K11" s="18" t="n">
+      <c r="K11" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="19" t="s">
         <v>150</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G12" s="18" t="s">
+      <c r="G12" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="H12" s="18" t="s">
+      <c r="H12" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="I12" s="18" t="n">
+      <c r="I12" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J12" s="18" t="n">
+      <c r="J12" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K12" s="18" t="n">
+      <c r="K12" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>153</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G13" s="18" t="s">
+      <c r="G13" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="H13" s="18" t="s">
+      <c r="H13" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="I13" s="18" t="n">
+      <c r="I13" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J13" s="18" t="n">
+      <c r="J13" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K13" s="18" t="n">
+      <c r="K13" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>155</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F14" s="18" t="s">
+      <c r="F14" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="G14" s="18" t="s">
+      <c r="G14" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="H14" s="18" t="s">
+      <c r="H14" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I14" s="18" t="n">
+      <c r="I14" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J14" s="18" t="n">
+      <c r="J14" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K14" s="18" t="n">
+      <c r="K14" s="19" t="n">
         <v>3</v>
       </c>
       <c r="L14" s="2"/>
-      <c r="XFD14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="19" t="s">
         <v>156</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>157</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="E15" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F15" s="18" t="s">
+      <c r="F15" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G15" s="18" t="s">
+      <c r="G15" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="H15" s="18" t="s">
+      <c r="H15" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="I15" s="18" t="n">
+      <c r="I15" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J15" s="18" t="n">
+      <c r="J15" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K15" s="18" t="n">
+      <c r="K15" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L15" s="2"/>
-      <c r="XFD15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F16" s="18" t="s">
+      <c r="F16" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G16" s="18" t="s">
+      <c r="G16" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="H16" s="18" t="s">
+      <c r="H16" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I16" s="18" t="n">
+      <c r="I16" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J16" s="18" t="n">
+      <c r="J16" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K16" s="18" t="n">
+      <c r="K16" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L16" s="2"/>
-      <c r="XFD16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F17" s="18" t="s">
+      <c r="F17" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G17" s="18" t="s">
+      <c r="G17" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="H17" s="18" t="s">
+      <c r="H17" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="I17" s="18" t="n">
+      <c r="I17" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J17" s="18" t="n">
+      <c r="J17" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K17" s="18" t="n">
+      <c r="K17" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L17" s="2"/>
-      <c r="XFD17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="19" t="s">
         <v>162</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F18" s="18" t="s">
+      <c r="F18" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G18" s="18" t="s">
+      <c r="G18" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="H18" s="18" t="s">
+      <c r="H18" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="I18" s="18" t="n">
+      <c r="I18" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J18" s="18" t="n">
+      <c r="J18" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K18" s="18" t="n">
+      <c r="K18" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L18" s="2"/>
-      <c r="XFD18" s="0"/>
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="19" t="s">
         <v>164</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="19" t="s">
         <v>165</v>
       </c>
       <c r="C19" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="E19" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="G19" s="18" t="s">
+      <c r="G19" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="H19" s="18" t="s">
+      <c r="H19" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I19" s="18" t="n">
+      <c r="I19" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J19" s="18" t="n">
+      <c r="J19" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K19" s="18" t="n">
+      <c r="K19" s="19" t="n">
         <v>3</v>
       </c>
       <c r="L19" s="2"/>
-      <c r="XFD19" s="0"/>
     </row>
     <row r="20" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="s">
+      <c r="A20" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="19" t="s">
         <v>167</v>
       </c>
       <c r="C20" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="E20" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F20" s="18" t="s">
+      <c r="F20" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G20" s="18" t="s">
+      <c r="G20" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="H20" s="18" t="s">
+      <c r="H20" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="I20" s="18" t="n">
+      <c r="I20" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J20" s="18" t="n">
+      <c r="J20" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K20" s="18" t="n">
+      <c r="K20" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L20" s="2"/>
-      <c r="XFD20" s="0"/>
     </row>
     <row r="21" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="19" t="s">
         <v>169</v>
       </c>
       <c r="C21" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="D21" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E21" s="18" t="s">
+      <c r="E21" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F21" s="18" t="s">
+      <c r="F21" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G21" s="18" t="s">
+      <c r="G21" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="H21" s="18" t="s">
+      <c r="H21" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I21" s="18" t="n">
+      <c r="I21" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J21" s="18" t="n">
+      <c r="J21" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K21" s="18" t="n">
+      <c r="K21" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L21" s="2"/>
-      <c r="XFD21" s="0"/>
     </row>
     <row r="22" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="19" t="s">
         <v>170</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="19" t="s">
         <v>171</v>
       </c>
       <c r="C22" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="D22" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E22" s="18" t="s">
+      <c r="E22" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G22" s="18" t="s">
+      <c r="G22" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="H22" s="18" t="s">
+      <c r="H22" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="I22" s="18" t="n">
+      <c r="I22" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J22" s="18" t="n">
+      <c r="J22" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K22" s="18" t="n">
+      <c r="K22" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L22" s="2"/>
-      <c r="XFD22" s="0"/>
     </row>
     <row r="23" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="19" t="s">
         <v>172</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="19" t="s">
         <v>173</v>
       </c>
       <c r="C23" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="D23" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E23" s="18" t="s">
+      <c r="E23" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F23" s="18" t="s">
+      <c r="F23" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G23" s="18" t="s">
+      <c r="G23" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="H23" s="18" t="s">
+      <c r="H23" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="I23" s="18" t="n">
+      <c r="I23" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J23" s="18" t="n">
+      <c r="J23" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K23" s="18" t="n">
+      <c r="K23" s="19" t="n">
         <v>10</v>
       </c>
       <c r="L23" s="2"/>
-      <c r="XFD23" s="0"/>
     </row>
     <row r="24" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="19" t="s">
         <v>175</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="E24" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F24" s="18" t="s">
+      <c r="F24" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="G24" s="18" t="s">
+      <c r="G24" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="H24" s="18" t="s">
+      <c r="H24" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I24" s="18" t="n">
+      <c r="I24" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J24" s="18" t="n">
+      <c r="J24" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K24" s="18" t="n">
+      <c r="K24" s="19" t="n">
         <v>3</v>
       </c>
       <c r="L24" s="2"/>
       <c r="XFD24" s="3"/>
     </row>
     <row r="25" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="19" t="s">
         <v>176</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="D25" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="E25" s="18" t="s">
+      <c r="E25" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F25" s="18" t="s">
+      <c r="F25" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="G25" s="18" t="s">
+      <c r="G25" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="H25" s="18" t="s">
+      <c r="H25" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I25" s="18" t="n">
+      <c r="I25" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J25" s="18" t="n">
+      <c r="J25" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K25" s="18" t="n">
+      <c r="K25" s="19" t="n">
         <v>3</v>
       </c>
       <c r="L25" s="2"/>
       <c r="XFD25" s="3"/>
     </row>
     <row r="26" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="19" t="s">
         <v>178</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="D26" s="18" t="s">
+      <c r="D26" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="E26" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F26" s="18" t="s">
+      <c r="F26" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="G26" s="18" t="s">
+      <c r="G26" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="H26" s="18" t="s">
+      <c r="H26" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="I26" s="18" t="n">
+      <c r="I26" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J26" s="18" t="n">
+      <c r="J26" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K26" s="18" t="n">
+      <c r="K26" s="19" t="n">
         <v>3</v>
       </c>
       <c r="L26" s="2"/>
@@ -4347,7 +4343,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.28"/>
@@ -4360,36 +4356,36 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>183</v>
       </c>
       <c r="XEV2" s="3"/>
@@ -4403,7 +4399,7 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>184</v>
       </c>
       <c r="B3" s="19" t="s">
@@ -4412,21 +4408,21 @@
       <c r="C3" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="18" t="n">
+      <c r="G3" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>187</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -4435,30 +4431,21 @@
       <c r="C4" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="18" t="n">
+      <c r="G4" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV4" s="0"/>
-      <c r="XEW4" s="0"/>
-      <c r="XEX4" s="0"/>
-      <c r="XEY4" s="0"/>
-      <c r="XEZ4" s="0"/>
-      <c r="XFA4" s="0"/>
-      <c r="XFB4" s="0"/>
-      <c r="XFC4" s="0"/>
-      <c r="XFD4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>189</v>
       </c>
       <c r="B5" s="19" t="s">
@@ -4467,30 +4454,21 @@
       <c r="C5" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="18" t="n">
+      <c r="G5" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV5" s="0"/>
-      <c r="XEW5" s="0"/>
-      <c r="XEX5" s="0"/>
-      <c r="XEY5" s="0"/>
-      <c r="XEZ5" s="0"/>
-      <c r="XFA5" s="0"/>
-      <c r="XFB5" s="0"/>
-      <c r="XFC5" s="0"/>
-      <c r="XFD5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>191</v>
       </c>
       <c r="B6" s="19" t="s">
@@ -4499,30 +4477,21 @@
       <c r="C6" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="18" t="n">
+      <c r="G6" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV6" s="0"/>
-      <c r="XEW6" s="0"/>
-      <c r="XEX6" s="0"/>
-      <c r="XEY6" s="0"/>
-      <c r="XEZ6" s="0"/>
-      <c r="XFA6" s="0"/>
-      <c r="XFB6" s="0"/>
-      <c r="XFC6" s="0"/>
-      <c r="XFD6" s="0"/>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>193</v>
       </c>
       <c r="B7" s="19" t="s">
@@ -4531,21 +4500,21 @@
       <c r="C7" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>195</v>
       </c>
       <c r="B8" s="19" t="s">
@@ -4554,30 +4523,21 @@
       <c r="C8" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="18" t="n">
+      <c r="G8" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV8" s="0"/>
-      <c r="XEW8" s="0"/>
-      <c r="XEX8" s="0"/>
-      <c r="XEY8" s="0"/>
-      <c r="XEZ8" s="0"/>
-      <c r="XFA8" s="0"/>
-      <c r="XFB8" s="0"/>
-      <c r="XFC8" s="0"/>
-      <c r="XFD8" s="0"/>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>197</v>
       </c>
       <c r="B9" s="19" t="s">
@@ -4586,30 +4546,21 @@
       <c r="C9" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="18" t="n">
+      <c r="G9" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV9" s="0"/>
-      <c r="XEW9" s="0"/>
-      <c r="XEX9" s="0"/>
-      <c r="XEY9" s="0"/>
-      <c r="XEZ9" s="0"/>
-      <c r="XFA9" s="0"/>
-      <c r="XFB9" s="0"/>
-      <c r="XFC9" s="0"/>
-      <c r="XFD9" s="0"/>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>199</v>
       </c>
       <c r="B10" s="19" t="s">
@@ -4618,30 +4569,21 @@
       <c r="C10" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="18" t="n">
+      <c r="G10" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV10" s="0"/>
-      <c r="XEW10" s="0"/>
-      <c r="XEX10" s="0"/>
-      <c r="XEY10" s="0"/>
-      <c r="XEZ10" s="0"/>
-      <c r="XFA10" s="0"/>
-      <c r="XFB10" s="0"/>
-      <c r="XFC10" s="0"/>
-      <c r="XFD10" s="0"/>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="19" t="s">
         <v>201</v>
       </c>
       <c r="B11" s="19" t="s">
@@ -4650,21 +4592,21 @@
       <c r="C11" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F11" s="18" t="n">
+      <c r="F11" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="18" t="n">
+      <c r="G11" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B12" s="19" t="s">
@@ -4673,30 +4615,21 @@
       <c r="C12" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F12" s="18" t="n">
+      <c r="F12" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="18" t="n">
+      <c r="G12" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV12" s="0"/>
-      <c r="XEW12" s="0"/>
-      <c r="XEX12" s="0"/>
-      <c r="XEY12" s="0"/>
-      <c r="XEZ12" s="0"/>
-      <c r="XFA12" s="0"/>
-      <c r="XFB12" s="0"/>
-      <c r="XFC12" s="0"/>
-      <c r="XFD12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="19" t="s">
         <v>205</v>
       </c>
       <c r="B13" s="19" t="s">
@@ -4705,30 +4638,21 @@
       <c r="C13" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="F13" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="G13" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV13" s="0"/>
-      <c r="XEW13" s="0"/>
-      <c r="XEX13" s="0"/>
-      <c r="XEY13" s="0"/>
-      <c r="XEZ13" s="0"/>
-      <c r="XFA13" s="0"/>
-      <c r="XFB13" s="0"/>
-      <c r="XFC13" s="0"/>
-      <c r="XFD13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="19" t="s">
         <v>207</v>
       </c>
       <c r="B14" s="19" t="s">
@@ -4737,30 +4661,21 @@
       <c r="C14" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F14" s="18" t="n">
+      <c r="F14" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G14" s="18" t="n">
+      <c r="G14" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV14" s="0"/>
-      <c r="XEW14" s="0"/>
-      <c r="XEX14" s="0"/>
-      <c r="XEY14" s="0"/>
-      <c r="XEZ14" s="0"/>
-      <c r="XFA14" s="0"/>
-      <c r="XFB14" s="0"/>
-      <c r="XFC14" s="0"/>
-      <c r="XFD14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="19" t="s">
         <v>209</v>
       </c>
       <c r="B15" s="19" t="s">
@@ -4769,21 +4684,21 @@
       <c r="C15" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F15" s="18" t="n">
+      <c r="F15" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="18" t="n">
+      <c r="G15" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="19" t="s">
         <v>211</v>
       </c>
       <c r="B16" s="19" t="s">
@@ -4792,30 +4707,21 @@
       <c r="C16" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E16" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F16" s="18" t="n">
+      <c r="F16" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="18" t="n">
+      <c r="G16" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV16" s="0"/>
-      <c r="XEW16" s="0"/>
-      <c r="XEX16" s="0"/>
-      <c r="XEY16" s="0"/>
-      <c r="XEZ16" s="0"/>
-      <c r="XFA16" s="0"/>
-      <c r="XFB16" s="0"/>
-      <c r="XFC16" s="0"/>
-      <c r="XFD16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="19" t="s">
         <v>213</v>
       </c>
       <c r="B17" s="19" t="s">
@@ -4824,30 +4730,21 @@
       <c r="C17" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E17" s="18" t="n">
+      <c r="E17" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F17" s="18" t="n">
+      <c r="F17" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="18" t="n">
+      <c r="G17" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV17" s="0"/>
-      <c r="XEW17" s="0"/>
-      <c r="XEX17" s="0"/>
-      <c r="XEY17" s="0"/>
-      <c r="XEZ17" s="0"/>
-      <c r="XFA17" s="0"/>
-      <c r="XFB17" s="0"/>
-      <c r="XFC17" s="0"/>
-      <c r="XFD17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="19" t="s">
         <v>215</v>
       </c>
       <c r="B18" s="19" t="s">
@@ -4856,27 +4753,18 @@
       <c r="C18" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E18" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F18" s="18" t="n">
+      <c r="F18" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G18" s="18" t="n">
+      <c r="G18" s="19" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV18" s="0"/>
-      <c r="XEW18" s="0"/>
-      <c r="XEX18" s="0"/>
-      <c r="XEY18" s="0"/>
-      <c r="XEZ18" s="0"/>
-      <c r="XFA18" s="0"/>
-      <c r="XFB18" s="0"/>
-      <c r="XFC18" s="0"/>
-      <c r="XFD18" s="0"/>
     </row>
     <row r="19" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -4909,12 +4797,12 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:R1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="2" width="26.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="34.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="34.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="35.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="28.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="28.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="64.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="29.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="12" width="51.08"/>
@@ -5020,28 +4908,28 @@
       <c r="E3" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="22" t="b">
+      <c r="F3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="G3" s="22" t="s">
         <v>234</v>
       </c>
-      <c r="H3" s="22" t="b">
+      <c r="H3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I3" s="22" t="s">
         <v>235</v>
       </c>
-      <c r="J3" s="22" t="b">
+      <c r="J3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K3" s="22" t="s">
         <v>236</v>
       </c>
-      <c r="L3" s="22" t="b">
+      <c r="L3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5080,28 +4968,28 @@
       <c r="E4" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="F4" s="22" t="b">
+      <c r="F4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="G4" s="22" t="s">
         <v>239</v>
       </c>
-      <c r="H4" s="22" t="b">
+      <c r="H4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I4" s="22" t="s">
         <v>240</v>
       </c>
-      <c r="J4" s="22" t="b">
+      <c r="J4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K4" s="22" t="s">
         <v>241</v>
       </c>
-      <c r="L4" s="22" t="b">
+      <c r="L4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5163,7 +5051,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD21"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="63.93"/>
@@ -5250,7 +5138,7 @@
       <c r="F3" s="22" t="s">
         <v>254</v>
       </c>
-      <c r="G3" s="22" t="b">
+      <c r="G3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5286,7 +5174,7 @@
       <c r="F4" s="22" t="s">
         <v>254</v>
       </c>
-      <c r="G4" s="22" t="b">
+      <c r="G4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5322,7 +5210,7 @@
       <c r="F5" s="22" t="s">
         <v>260</v>
       </c>
-      <c r="G5" s="22" t="b">
+      <c r="G5" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5358,7 +5246,7 @@
       <c r="F6" s="22" t="s">
         <v>260</v>
       </c>
-      <c r="G6" s="22" t="b">
+      <c r="G6" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5394,7 +5282,7 @@
       <c r="F7" s="22" t="s">
         <v>254</v>
       </c>
-      <c r="G7" s="22" t="b">
+      <c r="G7" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5430,7 +5318,7 @@
       <c r="F8" s="22" t="s">
         <v>260</v>
       </c>
-      <c r="G8" s="22" t="b">
+      <c r="G8" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Enable multi-agent PX4 launch
</commit_message>
<xml_diff>
--- a/config/Configuration-Test.xlsx
+++ b/config/Configuration-Test.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="281">
   <si>
     <t xml:space="preserve">GENERAL CONFIGURATION</t>
   </si>
@@ -94,27 +94,27 @@
     <t xml:space="preserve">(16:30:00)</t>
   </si>
   <si>
+    <t xml:space="preserve">MISSION01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single-Agent Test (Multi-Window)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISSION02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multi-Agent Test (Multi-Camera)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM02</t>
+  </si>
+  <si>
     <t xml:space="preserve">X</t>
   </si>
   <si>
-    <t xml:space="preserve">MISSION01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Single-Agent Test (Multi-Window)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAM01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multi-Agent Test (Multi-Camera)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAM02</t>
-  </si>
-  <si>
     <t xml:space="preserve">MISSION03</t>
   </si>
   <si>
@@ -292,16 +292,25 @@
     <t xml:space="preserve">TRACKING05</t>
   </si>
   <si>
+    <t xml:space="preserve">(X=10.0, Y=0.0, Z=0.0)</t>
+  </si>
+  <si>
     <t xml:space="preserve">AGENT06</t>
   </si>
   <si>
     <t xml:space="preserve">TRACKING06</t>
   </si>
   <si>
+    <t xml:space="preserve">(X=-10.0, Y=0.0, Z=0.0)</t>
+  </si>
+  <si>
     <t xml:space="preserve">AGENT07</t>
   </si>
   <si>
     <t xml:space="preserve">TRACKING07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(X=0.0, Y=10.0, Z=0.0)</t>
   </si>
   <si>
     <t xml:space="preserve">ObservationSetID</t>
@@ -938,18 +947,18 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="2" tint="-0.75"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1076,7 +1085,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1088,7 +1097,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1096,7 +1105,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1763,14 +1772,12 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="13"/>
+      <c r="B4" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="10" t="s">
         <v>22</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>23</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>13</v>
@@ -1779,7 +1786,7 @@
         <v>14</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G4" s="11" t="s">
         <v>16</v>
@@ -1845,10 +1852,10 @@
     <row r="5" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8"/>
       <c r="B5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>25</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>26</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>13</v>
@@ -1857,7 +1864,7 @@
         <v>14</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>16</v>
@@ -1921,7 +1928,9 @@
       <c r="BD5" s="12"/>
     </row>
     <row r="6" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8"/>
+      <c r="A6" s="8" t="s">
+        <v>27</v>
+      </c>
       <c r="B6" s="9" t="s">
         <v>28</v>
       </c>
@@ -2049,7 +2058,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -2070,62 +2079,62 @@
         <v>2</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="G2" s="21" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="H2" s="21" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="I2" s="21" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="J2" s="21" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="K2" s="21" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="E3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="G3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H3" s="22" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="I3" s="22" t="n">
         <v>0.4</v>
@@ -2715,7 +2724,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:XFD1048576"/>
+  <dimension ref="A1:XFD19"/>
   <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
@@ -2834,7 +2843,7 @@
         <v>75</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D4" s="19" t="s">
         <v>76</v>
@@ -2866,7 +2875,7 @@
         <v>78</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>79</v>
@@ -2898,7 +2907,7 @@
         <v>78</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>81</v>
@@ -2930,7 +2939,7 @@
         <v>78</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D7" s="19" t="s">
         <v>83</v>
@@ -2971,7 +2980,7 @@
         <v>71</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="G8" s="19" t="s">
         <v>73</v>
@@ -2988,7 +2997,7 @@
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>85</v>
@@ -2997,13 +3006,13 @@
         <v>30</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E9" s="19" t="s">
         <v>71</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="G9" s="19" t="s">
         <v>73</v>
@@ -3020,7 +3029,7 @@
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>85</v>
@@ -3029,13 +3038,13 @@
         <v>30</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E10" s="19" t="s">
         <v>71</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="G10" s="19" t="s">
         <v>73</v>
@@ -3059,7 +3068,6 @@
     <row r="17" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="18" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="19" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -3116,16 +3124,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H2" s="12"/>
       <c r="I2" s="12"/>
@@ -3144,10 +3152,10 @@
         <v>70</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D3" s="19" t="n">
         <v>0.2</v>
@@ -3169,10 +3177,10 @@
         <v>76</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D4" s="19" t="n">
         <v>0.2</v>
@@ -3194,10 +3202,10 @@
         <v>79</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D5" s="19" t="n">
         <v>0.2</v>
@@ -3219,10 +3227,10 @@
         <v>81</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D6" s="19" t="n">
         <v>0.2</v>
@@ -3244,10 +3252,10 @@
         <v>83</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D7" s="19" t="n">
         <v>0.2</v>
@@ -3269,10 +3277,10 @@
         <v>86</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D8" s="19" t="n">
         <v>0.2</v>
@@ -3291,13 +3299,13 @@
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D9" s="19" t="n">
         <v>0.2</v>
@@ -3316,13 +3324,13 @@
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D10" s="19" t="n">
         <v>0.2</v>
@@ -3374,7 +3382,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:XFD1048576"/>
+  <dimension ref="A1:XFD35"/>
   <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.34"/>
@@ -3412,16 +3420,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G2" s="18" t="s">
         <v>63</v>
@@ -3430,13 +3438,13 @@
         <v>64</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="K2" s="18" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="M2" s="12"/>
       <c r="N2" s="12"/>
@@ -3444,28 +3452,28 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G3" s="19" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H3" s="19" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I3" s="19" t="n">
         <v>3</v>
@@ -3480,28 +3488,28 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="I4" s="19" t="n">
         <v>8</v>
@@ -3516,28 +3524,28 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="F5" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="B5" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>96</v>
-      </c>
-      <c r="D5" s="19" t="s">
+      <c r="G5" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="H5" s="19" t="s">
         <v>126</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="F5" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="G5" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="H5" s="19" t="s">
-        <v>123</v>
       </c>
       <c r="I5" s="19" t="n">
         <v>8</v>
@@ -3552,28 +3560,28 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="H6" s="19" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I6" s="19" t="n">
         <v>8</v>
@@ -3588,28 +3596,28 @@
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="I7" s="19" t="n">
         <v>8</v>
@@ -3624,28 +3632,28 @@
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I8" s="19" t="n">
         <v>3</v>
@@ -3661,28 +3669,28 @@
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H9" s="19" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I9" s="19" t="n">
         <v>3</v>
@@ -3697,28 +3705,28 @@
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="I10" s="19" t="n">
         <v>8</v>
@@ -3733,28 +3741,28 @@
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D11" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="G11" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="H11" s="19" t="s">
         <v>126</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="F11" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="G11" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="H11" s="19" t="s">
-        <v>123</v>
       </c>
       <c r="I11" s="19" t="n">
         <v>8</v>
@@ -3769,28 +3777,28 @@
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="H12" s="19" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I12" s="19" t="n">
         <v>8</v>
@@ -3805,28 +3813,28 @@
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="H13" s="19" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="I13" s="19" t="n">
         <v>8</v>
@@ -3841,28 +3849,28 @@
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H14" s="19" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I14" s="19" t="n">
         <v>3</v>
@@ -3877,28 +3885,28 @@
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="I15" s="19" t="n">
         <v>8</v>
@@ -3913,28 +3921,28 @@
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D16" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="H16" s="19" t="s">
         <v>126</v>
-      </c>
-      <c r="E16" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="F16" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="G16" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="H16" s="19" t="s">
-        <v>123</v>
       </c>
       <c r="I16" s="19" t="n">
         <v>8</v>
@@ -3949,28 +3957,28 @@
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I17" s="19" t="n">
         <v>8</v>
@@ -3985,28 +3993,28 @@
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="H18" s="19" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="I18" s="19" t="n">
         <v>8</v>
@@ -4021,28 +4029,28 @@
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I19" s="19" t="n">
         <v>3</v>
@@ -4057,28 +4065,28 @@
     </row>
     <row r="20" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="H20" s="19" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="I20" s="19" t="n">
         <v>8</v>
@@ -4093,28 +4101,28 @@
     </row>
     <row r="21" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D21" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="E21" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="F21" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="G21" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="H21" s="19" t="s">
         <v>126</v>
-      </c>
-      <c r="E21" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="F21" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="G21" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="H21" s="19" t="s">
-        <v>123</v>
       </c>
       <c r="I21" s="19" t="n">
         <v>8</v>
@@ -4129,28 +4137,28 @@
     </row>
     <row r="22" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="H22" s="19" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I22" s="19" t="n">
         <v>8</v>
@@ -4165,28 +4173,28 @@
     </row>
     <row r="23" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="I23" s="19" t="n">
         <v>8</v>
@@ -4201,28 +4209,28 @@
     </row>
     <row r="24" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I24" s="19" t="n">
         <v>3</v>
@@ -4238,28 +4246,28 @@
     </row>
     <row r="25" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H25" s="19" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I25" s="19" t="n">
         <v>3</v>
@@ -4275,28 +4283,28 @@
     </row>
     <row r="26" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I26" s="19" t="n">
         <v>3</v>
@@ -4319,7 +4327,6 @@
     <row r="33" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="34" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="35" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -4374,19 +4381,19 @@
         <v>2</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="XEV2" s="3"/>
       <c r="XEW2" s="3"/>
@@ -4400,16 +4407,16 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E3" s="19" t="n">
         <v>0.167</v>
@@ -4423,16 +4430,16 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E4" s="19" t="n">
         <v>0.167</v>
@@ -4446,16 +4453,16 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5" s="19" t="s">
         <v>189</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>190</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>98</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>186</v>
       </c>
       <c r="E5" s="19" t="n">
         <v>0.167</v>
@@ -4469,16 +4476,16 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E6" s="19" t="n">
         <v>0.167</v>
@@ -4492,16 +4499,16 @@
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E7" s="19" t="n">
         <v>0.167</v>
@@ -4515,16 +4522,16 @@
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E8" s="19" t="n">
         <v>0.167</v>
@@ -4538,16 +4545,16 @@
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E9" s="19" t="n">
         <v>0.167</v>
@@ -4561,16 +4568,16 @@
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E10" s="19" t="n">
         <v>0.167</v>
@@ -4584,16 +4591,16 @@
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E11" s="19" t="n">
         <v>0.167</v>
@@ -4607,16 +4614,16 @@
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E12" s="19" t="n">
         <v>0.167</v>
@@ -4630,16 +4637,16 @@
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E13" s="19" t="n">
         <v>0.167</v>
@@ -4653,16 +4660,16 @@
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E14" s="19" t="n">
         <v>0.167</v>
@@ -4676,16 +4683,16 @@
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E15" s="19" t="n">
         <v>0.167</v>
@@ -4699,16 +4706,16 @@
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E16" s="19" t="n">
         <v>0.167</v>
@@ -4722,16 +4729,16 @@
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E17" s="19" t="n">
         <v>0.167</v>
@@ -4745,16 +4752,16 @@
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E18" s="19" t="n">
         <v>0.167</v>
@@ -4816,7 +4823,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -4847,49 +4854,49 @@
         <v>39</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="G2" s="21" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="H2" s="21" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="I2" s="21" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="J2" s="21" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="K2" s="21" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="L2" s="21" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="M2" s="21" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="N2" s="21" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="O2" s="21" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="P2" s="21" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="Q2" s="21" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="R2" s="21" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4900,7 +4907,7 @@
         <v>33</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D3" s="22" t="n">
         <v>8</v>
@@ -4913,28 +4920,28 @@
         <v>1</v>
       </c>
       <c r="G3" s="22" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="H3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I3" s="22" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="J3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K3" s="22" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="L3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="M3" s="22" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="N3" s="22" t="n">
         <v>6.5</v>
@@ -4954,13 +4961,13 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B4" s="22" t="s">
         <v>37</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D4" s="22" t="n">
         <v>8</v>
@@ -4973,28 +4980,28 @@
         <v>1</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I4" s="22" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="J4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K4" s="22" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="L4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="M4" s="22" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="N4" s="22" t="n">
         <v>6.5</v>
@@ -5068,7 +5075,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -5092,28 +5099,28 @@
         <v>39</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="G2" s="21" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="H2" s="21" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="I2" s="21" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="J2" s="21" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="K2" s="21" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="XFB2" s="3"/>
       <c r="XFC2" s="3"/>
@@ -5121,29 +5128,29 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="G3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H3" s="22" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I3" s="22" t="n">
         <v>0.5</v>
@@ -5157,29 +5164,29 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B4" s="22" t="s">
+        <v>259</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>254</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="E4" s="22" t="s">
         <v>256</v>
       </c>
-      <c r="C4" s="22" t="s">
-        <v>251</v>
-      </c>
-      <c r="D4" s="22" t="s">
+      <c r="F4" s="22" t="s">
         <v>257</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>253</v>
-      </c>
-      <c r="F4" s="22" t="s">
-        <v>254</v>
       </c>
       <c r="G4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H4" s="22" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I4" s="22" t="n">
         <v>0.5</v>
@@ -5193,29 +5200,29 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="G5" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H5" s="22" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="I5" s="22" t="n">
         <v>0.5</v>
@@ -5229,29 +5236,29 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B6" s="22" t="s">
+        <v>266</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>254</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>256</v>
+      </c>
+      <c r="F6" s="22" t="s">
         <v>263</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>251</v>
-      </c>
-      <c r="D6" s="22" t="s">
-        <v>257</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>253</v>
-      </c>
-      <c r="F6" s="22" t="s">
-        <v>260</v>
       </c>
       <c r="G6" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H6" s="22" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="I6" s="22" t="n">
         <v>0.5</v>
@@ -5265,29 +5272,29 @@
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="G7" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H7" s="22" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I7" s="22" t="n">
         <v>0.8</v>
@@ -5301,29 +5308,29 @@
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="G8" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="I8" s="22" t="n">
         <v>0.8</v>

</xml_diff>

<commit_message>
Setup mavROS frame convention
</commit_message>
<xml_diff>
--- a/config/Configuration-Test.xlsx
+++ b/config/Configuration-Test.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -139,35 +139,7 @@
     <t xml:space="preserve">MISSION05</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Multi-Agent Test (Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">Multi-Agent Test (Multi-Hybrid)</t>
   </si>
   <si>
     <t xml:space="preserve">TEAM05</t>
@@ -455,69 +427,13 @@
     <t xml:space="preserve">SET09</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Tracking 2 (Multi)</t>
-    </r>
+    <t xml:space="preserve">Multi-Hybrid Tracking 2 (Multi)</t>
   </si>
   <si>
     <t xml:space="preserve">SET10</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Tracking 3 (Multi)</t>
-    </r>
+    <t xml:space="preserve">Multi-Hybrid Tracking 3 (Multi)</t>
   </si>
   <si>
     <t xml:space="preserve">SET11</t>
@@ -634,69 +550,13 @@
     <t xml:space="preserve">MULTICAMERA7</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Head 1 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (Single)</t>
-    </r>
+    <t xml:space="preserve">Tracking Head 1 Multi-Hybrid (Single)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA8</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Head 2 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (Single)</t>
-    </r>
+    <t xml:space="preserve">Tracking Head 2 Multi-Hybrid (Single)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA9</t>
@@ -780,107 +640,13 @@
     <t xml:space="preserve">MULTICAMERA22</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Head 1 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 1 (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Multi</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">Tracking Head 1 Multi-Hybrid 1 (Multi)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA23</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Head 2 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 1 (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Multi</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">Tracking Head 2 Multi-Hybrid 1 (Multi)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA24</t>
@@ -892,107 +658,13 @@
     <t xml:space="preserve">MULTICAMERA25</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Head 1 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 2 (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Multi</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">Tracking Head 1 Multi-Hybrid 2 (Multi)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA26</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Head 2 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 2 (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Multi</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">Tracking Head 2 Multi-Hybrid 2 (Multi)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA27</t>
@@ -1004,107 +676,13 @@
     <t xml:space="preserve">MULTICAMERA28</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Head 1 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 3 (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Multi</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">Tracking Head 1 Multi-Hybrid 3 (Multi)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA29</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Head 2 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid 3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Multi</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">Tracking Head 2 Multi-Hybrid 3 (Multi)</t>
   </si>
   <si>
     <t xml:space="preserve">Resolution [pix]</t>
@@ -1155,35 +733,7 @@
     <t xml:space="preserve">MULTIWINDOW05</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Window 2 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (Single)</t>
-    </r>
+    <t xml:space="preserve">Tracking Window 2 Multi-Hybrid (Single)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTIWINDOW06</t>
@@ -1231,35 +781,7 @@
     <t xml:space="preserve">MULTIWINDOW13</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Window 2 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid 1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (Multi)</t>
-    </r>
+    <t xml:space="preserve">Tracking Window 2 Multi-Hybrid 1 (Multi)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTIWINDOW14</t>
@@ -1271,35 +793,7 @@
     <t xml:space="preserve">MULTIWINDOW15</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Window 2 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid 2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (Multi)</t>
-    </r>
+    <t xml:space="preserve">Tracking Window 2 Multi-Hybrid 2 (Multi)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTIWINDOW16</t>
@@ -1311,35 +805,7 @@
     <t xml:space="preserve">MULTIWINDOW17</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tracking Window 2 Multi-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Hybrid 3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (Multi)</t>
-    </r>
+    <t xml:space="preserve">Tracking Window 2 Multi-Hybrid 3 (Multi)</t>
   </si>
   <si>
     <t xml:space="preserve">HARDWARE CATALOGS</t>
@@ -1529,13 +995,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0"/>
-    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="10">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1603,19 +1068,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1709,7 +1161,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1762,10 +1214,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1799,10 +1247,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2286,7 +1730,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="21" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="21" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.44"/>
@@ -2429,7 +1873,7 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="8" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="9" t="s">
@@ -2509,7 +1953,7 @@
       <c r="BD4" s="12"/>
     </row>
     <row r="5" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13"/>
+      <c r="A5" s="8"/>
       <c r="B5" s="9" t="s">
         <v>25</v>
       </c>
@@ -2585,8 +2029,6 @@
       <c r="BB5" s="12"/>
       <c r="BC5" s="12"/>
       <c r="BD5" s="12"/>
-      <c r="XFC5" s="0"/>
-      <c r="XFD5" s="0"/>
     </row>
     <row r="6" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8"/>
@@ -2856,7 +2298,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD16"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="2" width="29.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="40.25"/>
@@ -2870,92 +2312,92 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>259</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>310</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>311</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>312</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>313</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>314</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>315</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>289</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>290</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>291</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>316</v>
       </c>
-      <c r="C3" s="23" t="b">
+      <c r="C3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="21" t="s">
         <v>317</v>
       </c>
-      <c r="E3" s="23" t="b">
+      <c r="E3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="21" t="s">
         <v>318</v>
       </c>
-      <c r="G3" s="23" t="b">
+      <c r="G3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="21" t="s">
         <v>319</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="21" t="n">
         <v>0.4</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="21" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2995,7 +2437,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="33.54"/>
@@ -3008,12 +2450,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -3043,7 +2485,7 @@
       <c r="C3" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="14" t="s">
         <v>42</v>
       </c>
     </row>
@@ -3057,7 +2499,7 @@
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="14" t="s">
         <v>45</v>
       </c>
     </row>
@@ -3086,7 +2528,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:BM1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="38.38"/>
@@ -3097,15 +2539,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -3201,7 +2643,7 @@
       <c r="D3" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="15" t="n">
         <v>2</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -3282,7 +2724,7 @@
       <c r="D4" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="E4" s="15" t="n">
         <v>4</v>
       </c>
       <c r="F4" s="9" t="s">
@@ -3363,7 +2805,7 @@
       <c r="D5" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="15" t="n">
         <v>8</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -3444,7 +2886,7 @@
       <c r="D6" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="15" t="n">
         <v>16</v>
       </c>
       <c r="F6" s="9" t="s">
@@ -3538,7 +2980,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD20"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -3557,50 +2999,50 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
       <c r="XFC1" s="3"/>
       <c r="XFD1" s="3"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>73</v>
       </c>
       <c r="L2" s="12"/>
@@ -3615,390 +3057,390 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="19" t="n">
+      <c r="H3" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="J3" s="18" t="n">
         <v>12000</v>
       </c>
       <c r="XFC3" s="3"/>
       <c r="XFD3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H4" s="19" t="n">
+      <c r="H4" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="19" t="n">
+      <c r="I4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="19" t="n">
+      <c r="J4" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H5" s="19" t="n">
+      <c r="H5" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="19" t="n">
+      <c r="J5" s="18" t="n">
         <v>12000</v>
       </c>
-      <c r="XFC5" s="0"/>
-      <c r="XFD5" s="0"/>
+      <c r="XFC5" s="3"/>
+      <c r="XFD5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H6" s="19" t="n">
+      <c r="H6" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="J6" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="19" t="n">
+      <c r="H7" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="J7" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="H8" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="J8" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="H9" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="19" t="n">
+      <c r="H11" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I11" s="19" t="n">
+      <c r="I11" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J11" s="19" t="n">
+      <c r="J11" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H12" s="19" t="n">
+      <c r="H12" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I12" s="19" t="n">
+      <c r="I12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J12" s="19" t="n">
+      <c r="J12" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H13" s="19" t="n">
+      <c r="H13" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I13" s="19" t="n">
+      <c r="I13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J13" s="19" t="n">
+      <c r="J13" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H14" s="19" t="n">
+      <c r="H14" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I14" s="19" t="n">
+      <c r="I14" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J14" s="19" t="n">
+      <c r="J14" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -4031,7 +3473,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD24"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -4047,32 +3489,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>111</v>
       </c>
       <c r="H2" s="12"/>
@@ -4088,22 +3530,22 @@
       <c r="XFD2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D3" s="19" t="n">
+      <c r="D3" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G3" s="2"/>
@@ -4113,22 +3555,22 @@
       <c r="XEY3" s="3"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D4" s="19" t="n">
+      <c r="D4" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G4" s="2"/>
@@ -4138,22 +3580,22 @@
       <c r="XEY4" s="3"/>
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G5" s="2"/>
@@ -4161,29 +3603,29 @@
       <c r="XEW5" s="2"/>
       <c r="XEX5" s="2"/>
       <c r="XEY5" s="3"/>
-      <c r="XEZ5" s="0"/>
-      <c r="XFA5" s="0"/>
-      <c r="XFB5" s="0"/>
-      <c r="XFC5" s="0"/>
-      <c r="XFD5" s="0"/>
+      <c r="XEZ5" s="3"/>
+      <c r="XFA5" s="3"/>
+      <c r="XFB5" s="3"/>
+      <c r="XFC5" s="3"/>
+      <c r="XFD5" s="3"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G6" s="2"/>
@@ -4193,22 +3635,22 @@
       <c r="XEY6" s="3"/>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G7" s="2"/>
@@ -4218,22 +3660,22 @@
       <c r="XEY7" s="3"/>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G8" s="2"/>
@@ -4243,22 +3685,22 @@
       <c r="XEY8" s="3"/>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G9" s="2"/>
@@ -4268,22 +3710,22 @@
       <c r="XEY9" s="3"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G10" s="2"/>
@@ -4293,22 +3735,22 @@
       <c r="XEY10" s="3"/>
     </row>
     <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>128</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F11" s="19" t="n">
+      <c r="F11" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G11" s="2"/>
@@ -4318,22 +3760,22 @@
       <c r="XEY11" s="3"/>
     </row>
     <row r="12" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="D12" s="19" t="n">
+      <c r="D12" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E12" s="19" t="n">
+      <c r="E12" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F12" s="19" t="n">
+      <c r="F12" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G12" s="2"/>
@@ -4343,22 +3785,22 @@
       <c r="XEY12" s="3"/>
     </row>
     <row r="13" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="D13" s="19" t="n">
+      <c r="D13" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E13" s="19" t="n">
+      <c r="E13" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F13" s="19" t="n">
+      <c r="F13" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G13" s="2"/>
@@ -4368,22 +3810,22 @@
       <c r="XEY13" s="3"/>
     </row>
     <row r="14" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E14" s="19" t="n">
+      <c r="E14" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F14" s="19" t="n">
+      <c r="F14" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G14" s="2"/>
@@ -4425,7 +3867,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD32"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.28"/>
@@ -4439,53 +3881,53 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
       <c r="L1" s="2"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>138</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="17" t="s">
         <v>142</v>
       </c>
       <c r="M2" s="12"/>
@@ -4493,1086 +3935,1085 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="J3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="19" t="n">
+      <c r="K3" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H4" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="I4" s="19" t="n">
+      <c r="I4" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J4" s="19" t="n">
+      <c r="J4" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="19" t="n">
+      <c r="K4" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J5" s="19" t="n">
+      <c r="J5" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K5" s="19" t="n">
+      <c r="K5" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="J6" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K6" s="19" t="n">
+      <c r="K6" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>165</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="H7" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="J7" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K7" s="19" t="n">
+      <c r="K7" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L7" s="2"/>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="J8" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="K8" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L8" s="2"/>
       <c r="XFD8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="K9" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="H10" s="19" t="s">
+      <c r="H10" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K10" s="19" t="n">
+      <c r="K10" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="H11" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I11" s="19" t="n">
+      <c r="I11" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J11" s="19" t="n">
+      <c r="J11" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="K11" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H12" s="19" t="s">
+      <c r="H12" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I12" s="19" t="n">
+      <c r="I12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J12" s="19" t="n">
+      <c r="J12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K12" s="19" t="n">
+      <c r="K12" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L12" s="2"/>
-      <c r="XFD12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="H13" s="19" t="s">
+      <c r="H13" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="I13" s="19" t="n">
+      <c r="I13" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J13" s="19" t="n">
+      <c r="J13" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K13" s="19" t="n">
+      <c r="K13" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I14" s="19" t="n">
+      <c r="I14" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J14" s="19" t="n">
+      <c r="J14" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K14" s="19" t="n">
+      <c r="K14" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F15" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H15" s="19" t="s">
+      <c r="H15" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I15" s="19" t="n">
+      <c r="I15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J15" s="19" t="n">
+      <c r="J15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K15" s="19" t="n">
+      <c r="K15" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="G16" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="H16" s="19" t="s">
+      <c r="H16" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="I16" s="19" t="n">
+      <c r="I16" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J16" s="19" t="n">
+      <c r="J16" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K16" s="19" t="n">
+      <c r="K16" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D17" s="19" t="s">
+      <c r="D17" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="E17" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="F17" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="H17" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I17" s="19" t="n">
+      <c r="I17" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J17" s="19" t="n">
+      <c r="J17" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K17" s="19" t="n">
+      <c r="K17" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="E18" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="F18" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G18" s="19" t="s">
+      <c r="G18" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H18" s="19" t="s">
+      <c r="H18" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I18" s="19" t="n">
+      <c r="I18" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J18" s="19" t="n">
+      <c r="J18" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K18" s="19" t="n">
+      <c r="K18" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="D19" s="19" t="s">
+      <c r="D19" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E19" s="19" t="s">
+      <c r="E19" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F19" s="19" t="s">
+      <c r="F19" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G19" s="19" t="s">
+      <c r="G19" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="H19" s="19" t="s">
+      <c r="H19" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="I19" s="19" t="n">
+      <c r="I19" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J19" s="19" t="n">
+      <c r="J19" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K19" s="19" t="n">
+      <c r="K19" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="C20" s="19" t="s">
+      <c r="C20" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="D20" s="19" t="s">
+      <c r="D20" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E20" s="19" t="s">
+      <c r="E20" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F20" s="19" t="s">
+      <c r="F20" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G20" s="19" t="s">
+      <c r="G20" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="H20" s="19" t="s">
+      <c r="H20" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I20" s="19" t="n">
+      <c r="I20" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J20" s="19" t="n">
+      <c r="J20" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K20" s="19" t="n">
+      <c r="K20" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L20" s="2"/>
     </row>
     <row r="21" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="C21" s="19" t="s">
+      <c r="C21" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="D21" s="19" t="s">
+      <c r="D21" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="E21" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F21" s="19" t="s">
+      <c r="F21" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H21" s="19" t="s">
+      <c r="H21" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I21" s="19" t="n">
+      <c r="I21" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J21" s="19" t="n">
+      <c r="J21" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K21" s="19" t="n">
+      <c r="K21" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L21" s="2"/>
       <c r="XFD21" s="3"/>
     </row>
     <row r="22" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="C22" s="19" t="s">
+      <c r="C22" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="D22" s="19" t="s">
+      <c r="D22" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="E22" s="19" t="s">
+      <c r="E22" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F22" s="19" t="s">
+      <c r="F22" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H22" s="19" t="s">
+      <c r="H22" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I22" s="19" t="n">
+      <c r="I22" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J22" s="19" t="n">
+      <c r="J22" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K22" s="19" t="n">
+      <c r="K22" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L22" s="2"/>
       <c r="XFD22" s="3"/>
     </row>
     <row r="23" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="18" t="s">
         <v>198</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="C23" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D23" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="E23" s="19" t="s">
+      <c r="E23" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F23" s="19" t="s">
+      <c r="F23" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G23" s="19" t="s">
+      <c r="G23" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H23" s="19" t="s">
+      <c r="H23" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I23" s="19" t="n">
+      <c r="I23" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J23" s="19" t="n">
+      <c r="J23" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K23" s="19" t="n">
+      <c r="K23" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L23" s="2"/>
       <c r="XFD23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="C24" s="19" t="s">
+      <c r="C24" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="D24" s="19" t="s">
+      <c r="D24" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="E24" s="19" t="s">
+      <c r="E24" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F24" s="19" t="s">
+      <c r="F24" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G24" s="19" t="s">
+      <c r="G24" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H24" s="19" t="s">
+      <c r="H24" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I24" s="19" t="n">
+      <c r="I24" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J24" s="19" t="n">
+      <c r="J24" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K24" s="19" t="n">
+      <c r="K24" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
+      <c r="A25" s="18" t="s">
         <v>202</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="C25" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="D25" s="19" t="s">
+      <c r="D25" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E25" s="19" t="s">
+      <c r="E25" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F25" s="19" t="s">
+      <c r="F25" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G25" s="19" t="s">
+      <c r="G25" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="H25" s="19" t="s">
+      <c r="H25" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="I25" s="19" t="n">
+      <c r="I25" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J25" s="19" t="n">
+      <c r="J25" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K25" s="19" t="n">
+      <c r="K25" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19" t="s">
+      <c r="A26" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="B26" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="C26" s="19" t="s">
+      <c r="C26" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="D26" s="19" t="s">
+      <c r="D26" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E26" s="19" t="s">
+      <c r="E26" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F26" s="19" t="s">
+      <c r="F26" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G26" s="19" t="s">
+      <c r="G26" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="H26" s="19" t="s">
+      <c r="H26" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I26" s="19" t="n">
+      <c r="I26" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J26" s="19" t="n">
+      <c r="J26" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K26" s="19" t="n">
+      <c r="K26" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="18" t="s">
         <v>207</v>
       </c>
-      <c r="C27" s="19" t="s">
+      <c r="C27" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="D27" s="19" t="s">
+      <c r="D27" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="E27" s="19" t="s">
+      <c r="E27" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F27" s="19" t="s">
+      <c r="F27" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G27" s="19" t="s">
+      <c r="G27" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H27" s="19" t="s">
+      <c r="H27" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I27" s="19" t="n">
+      <c r="I27" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J27" s="19" t="n">
+      <c r="J27" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K27" s="19" t="n">
+      <c r="K27" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="18" t="s">
         <v>208</v>
       </c>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="18" t="s">
         <v>209</v>
       </c>
-      <c r="C28" s="19" t="s">
+      <c r="C28" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="D28" s="19" t="s">
+      <c r="D28" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E28" s="19" t="s">
+      <c r="E28" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F28" s="19" t="s">
+      <c r="F28" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G28" s="19" t="s">
+      <c r="G28" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="H28" s="19" t="s">
+      <c r="H28" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="I28" s="19" t="n">
+      <c r="I28" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J28" s="19" t="n">
+      <c r="J28" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K28" s="19" t="n">
+      <c r="K28" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="s">
+      <c r="A29" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="C29" s="19" t="s">
+      <c r="C29" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="D29" s="19" t="s">
+      <c r="D29" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E29" s="19" t="s">
+      <c r="E29" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F29" s="19" t="s">
+      <c r="F29" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G29" s="19" t="s">
+      <c r="G29" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="H29" s="19" t="s">
+      <c r="H29" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I29" s="19" t="n">
+      <c r="I29" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J29" s="19" t="n">
+      <c r="J29" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K29" s="19" t="n">
+      <c r="K29" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="18" t="s">
         <v>212</v>
       </c>
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="18" t="s">
         <v>213</v>
       </c>
-      <c r="C30" s="19" t="s">
+      <c r="C30" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="D30" s="19" t="s">
+      <c r="D30" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="E30" s="19" t="s">
+      <c r="E30" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F30" s="19" t="s">
+      <c r="F30" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G30" s="19" t="s">
+      <c r="G30" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H30" s="19" t="s">
+      <c r="H30" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I30" s="19" t="n">
+      <c r="I30" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J30" s="19" t="n">
+      <c r="J30" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K30" s="19" t="n">
+      <c r="K30" s="18" t="n">
         <v>3</v>
       </c>
       <c r="L30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="19" t="s">
+      <c r="A31" s="18" t="s">
         <v>214</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="18" t="s">
         <v>215</v>
       </c>
-      <c r="C31" s="19" t="s">
+      <c r="C31" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="D31" s="19" t="s">
+      <c r="D31" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E31" s="19" t="s">
+      <c r="E31" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F31" s="19" t="s">
+      <c r="F31" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G31" s="19" t="s">
+      <c r="G31" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="H31" s="19" t="s">
+      <c r="H31" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="I31" s="19" t="n">
+      <c r="I31" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J31" s="19" t="n">
+      <c r="J31" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K31" s="19" t="n">
+      <c r="K31" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="19" t="s">
+      <c r="A32" s="18" t="s">
         <v>216</v>
       </c>
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="18" t="s">
         <v>217</v>
       </c>
-      <c r="C32" s="19" t="s">
+      <c r="C32" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="D32" s="19" t="s">
+      <c r="D32" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E32" s="19" t="s">
+      <c r="E32" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F32" s="19" t="s">
+      <c r="F32" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G32" s="19" t="s">
+      <c r="G32" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="H32" s="19" t="s">
+      <c r="H32" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="I32" s="19" t="n">
+      <c r="I32" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="J32" s="19" t="n">
+      <c r="J32" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K32" s="19" t="n">
+      <c r="K32" s="18" t="n">
         <v>10</v>
       </c>
       <c r="L32" s="2"/>
@@ -5600,7 +5041,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD20"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.28"/>
@@ -5613,36 +5054,36 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>218</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>219</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>220</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>221</v>
       </c>
       <c r="XEV2" s="3"/>
@@ -5656,490 +5097,418 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>222</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="19" t="n">
+      <c r="G3" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>225</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="19" t="n">
+      <c r="G4" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>227</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>228</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="19" t="n">
+      <c r="G5" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>229</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="19" t="n">
+      <c r="G6" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>231</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>232</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="G7" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV7" s="0"/>
-      <c r="XEW7" s="0"/>
-      <c r="XEX7" s="0"/>
-      <c r="XEY7" s="0"/>
-      <c r="XEZ7" s="0"/>
-      <c r="XFA7" s="0"/>
-      <c r="XFB7" s="0"/>
-      <c r="XFC7" s="0"/>
-      <c r="XFD7" s="0"/>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>233</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>234</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="G8" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV8" s="0"/>
-      <c r="XEW8" s="0"/>
-      <c r="XEX8" s="0"/>
-      <c r="XEY8" s="0"/>
-      <c r="XEZ8" s="0"/>
-      <c r="XFA8" s="0"/>
-      <c r="XFB8" s="0"/>
-      <c r="XFC8" s="0"/>
-      <c r="XFD8" s="0"/>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>235</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>238</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>239</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>240</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F11" s="19" t="n">
+      <c r="F11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="18" t="s">
         <v>241</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>242</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E12" s="19" t="n">
+      <c r="E12" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F12" s="19" t="n">
+      <c r="F12" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="19" t="n">
+      <c r="G12" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>243</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="18" t="s">
         <v>244</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E13" s="19" t="n">
+      <c r="E13" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F13" s="19" t="n">
+      <c r="F13" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G13" s="19" t="n">
+      <c r="G13" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="18" t="s">
         <v>245</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="18" t="s">
         <v>246</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E14" s="19" t="n">
+      <c r="E14" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F14" s="19" t="n">
+      <c r="F14" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G14" s="19" t="n">
+      <c r="G14" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="18" t="s">
         <v>247</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E15" s="19" t="n">
+      <c r="E15" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F15" s="19" t="n">
+      <c r="F15" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="19" t="n">
+      <c r="G15" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV15" s="0"/>
-      <c r="XEW15" s="0"/>
-      <c r="XEX15" s="0"/>
-      <c r="XEY15" s="0"/>
-      <c r="XEZ15" s="0"/>
-      <c r="XFA15" s="0"/>
-      <c r="XFB15" s="0"/>
-      <c r="XFC15" s="0"/>
-      <c r="XFD15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="18" t="s">
         <v>249</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="18" t="s">
         <v>250</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E16" s="19" t="n">
+      <c r="E16" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F16" s="19" t="n">
+      <c r="F16" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="19" t="n">
+      <c r="G16" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV16" s="0"/>
-      <c r="XEW16" s="0"/>
-      <c r="XEX16" s="0"/>
-      <c r="XEY16" s="0"/>
-      <c r="XEZ16" s="0"/>
-      <c r="XFA16" s="0"/>
-      <c r="XFB16" s="0"/>
-      <c r="XFC16" s="0"/>
-      <c r="XFD16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="18" t="s">
         <v>251</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="18" t="s">
         <v>252</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="D17" s="19" t="s">
+      <c r="D17" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E17" s="19" t="n">
+      <c r="E17" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F17" s="19" t="n">
+      <c r="F17" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="19" t="n">
+      <c r="G17" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV17" s="0"/>
-      <c r="XEW17" s="0"/>
-      <c r="XEX17" s="0"/>
-      <c r="XEY17" s="0"/>
-      <c r="XEZ17" s="0"/>
-      <c r="XFA17" s="0"/>
-      <c r="XFB17" s="0"/>
-      <c r="XFC17" s="0"/>
-      <c r="XFD17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="18" t="s">
         <v>253</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="18" t="s">
         <v>254</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E18" s="19" t="n">
+      <c r="E18" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F18" s="19" t="n">
+      <c r="F18" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G18" s="19" t="n">
+      <c r="G18" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV18" s="0"/>
-      <c r="XEW18" s="0"/>
-      <c r="XEX18" s="0"/>
-      <c r="XEY18" s="0"/>
-      <c r="XEZ18" s="0"/>
-      <c r="XFA18" s="0"/>
-      <c r="XFB18" s="0"/>
-      <c r="XFC18" s="0"/>
-      <c r="XFD18" s="0"/>
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="18" t="s">
         <v>255</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="18" t="s">
         <v>256</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="D19" s="19" t="s">
+      <c r="D19" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E19" s="19" t="n">
+      <c r="E19" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F19" s="19" t="n">
+      <c r="F19" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="19" t="n">
+      <c r="G19" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV19" s="0"/>
-      <c r="XEW19" s="0"/>
-      <c r="XEX19" s="0"/>
-      <c r="XEY19" s="0"/>
-      <c r="XEZ19" s="0"/>
-      <c r="XFA19" s="0"/>
-      <c r="XFB19" s="0"/>
-      <c r="XFC19" s="0"/>
-      <c r="XFD19" s="0"/>
     </row>
     <row r="20" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="18" t="s">
         <v>257</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="18" t="s">
         <v>258</v>
       </c>
-      <c r="C20" s="19" t="s">
+      <c r="C20" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="D20" s="19" t="s">
+      <c r="D20" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E20" s="19" t="n">
+      <c r="E20" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F20" s="19" t="n">
+      <c r="F20" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="19" t="n">
+      <c r="G20" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="XEV20" s="0"/>
-      <c r="XEW20" s="0"/>
-      <c r="XEX20" s="0"/>
-      <c r="XEY20" s="0"/>
-      <c r="XEZ20" s="0"/>
-      <c r="XFA20" s="0"/>
-      <c r="XFB20" s="0"/>
-      <c r="XFC20" s="0"/>
-      <c r="XFD20" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6164,7 +5533,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:R1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="34.63"/>
@@ -6182,200 +5551,200 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>259</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>260</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>261</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>263</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>266</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>267</v>
       </c>
-      <c r="L2" s="21" t="s">
+      <c r="L2" s="20" t="s">
         <v>268</v>
       </c>
-      <c r="M2" s="21" t="s">
+      <c r="M2" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="N2" s="21" t="s">
+      <c r="N2" s="20" t="s">
         <v>270</v>
       </c>
-      <c r="O2" s="21" t="s">
+      <c r="O2" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="P2" s="21" t="s">
+      <c r="P2" s="20" t="s">
         <v>272</v>
       </c>
-      <c r="Q2" s="21" t="s">
+      <c r="Q2" s="20" t="s">
         <v>273</v>
       </c>
-      <c r="R2" s="21" t="s">
+      <c r="R2" s="20" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>275</v>
       </c>
-      <c r="D3" s="22" t="n">
+      <c r="D3" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="22" t="n">
+      <c r="E3" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="23" t="b">
+      <c r="F3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="21" t="s">
         <v>276</v>
       </c>
-      <c r="H3" s="23" t="b">
+      <c r="H3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="I3" s="22" t="s">
+      <c r="I3" s="21" t="s">
         <v>277</v>
       </c>
-      <c r="J3" s="23" t="b">
+      <c r="J3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K3" s="22" t="s">
+      <c r="K3" s="21" t="s">
         <v>278</v>
       </c>
-      <c r="L3" s="23" t="b">
+      <c r="L3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="M3" s="22" t="s">
+      <c r="M3" s="21" t="s">
         <v>279</v>
       </c>
-      <c r="N3" s="22" t="n">
+      <c r="N3" s="21" t="n">
         <v>6.5</v>
       </c>
-      <c r="O3" s="22" t="n">
+      <c r="O3" s="21" t="n">
         <v>2.5</v>
       </c>
-      <c r="P3" s="22" t="n">
+      <c r="P3" s="21" t="n">
         <v>400</v>
       </c>
-      <c r="Q3" s="22" t="n">
+      <c r="Q3" s="21" t="n">
         <v>350</v>
       </c>
-      <c r="R3" s="22" t="n">
+      <c r="R3" s="21" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>280</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="21" t="s">
         <v>275</v>
       </c>
-      <c r="D4" s="22" t="n">
+      <c r="D4" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="22" t="n">
+      <c r="E4" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F4" s="23" t="b">
+      <c r="F4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="G4" s="21" t="s">
         <v>281</v>
       </c>
-      <c r="H4" s="23" t="b">
+      <c r="H4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="I4" s="22" t="s">
+      <c r="I4" s="21" t="s">
         <v>282</v>
       </c>
-      <c r="J4" s="23" t="b">
+      <c r="J4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K4" s="22" t="s">
+      <c r="K4" s="21" t="s">
         <v>283</v>
       </c>
-      <c r="L4" s="23" t="b">
+      <c r="L4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="M4" s="22" t="s">
+      <c r="M4" s="21" t="s">
         <v>284</v>
       </c>
-      <c r="N4" s="22" t="n">
+      <c r="N4" s="21" t="n">
         <v>6.5</v>
       </c>
-      <c r="O4" s="22" t="n">
+      <c r="O4" s="21" t="n">
         <v>2.5</v>
       </c>
-      <c r="P4" s="22" t="n">
+      <c r="P4" s="21" t="n">
         <v>400</v>
       </c>
-      <c r="Q4" s="22" t="n">
+      <c r="Q4" s="21" t="n">
         <v>350</v>
       </c>
-      <c r="R4" s="22" t="n">
+      <c r="R4" s="21" t="n">
         <v>25</v>
       </c>
     </row>
@@ -6418,7 +5787,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD21"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="63.93"/>
@@ -6434,52 +5803,52 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>259</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>285</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>286</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>287</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>288</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>289</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>290</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>291</v>
       </c>
       <c r="XFB2" s="3"/>
@@ -6487,218 +5856,218 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>292</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="21" t="s">
         <v>294</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="21" t="s">
         <v>296</v>
       </c>
-      <c r="G3" s="23" t="b">
+      <c r="G3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>298</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>299</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="21" t="s">
         <v>296</v>
       </c>
-      <c r="G4" s="23" t="b">
+      <c r="G4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="I4" s="22" t="n">
+      <c r="I4" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="J4" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="22" t="n">
+      <c r="K4" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>300</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>301</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="21" t="s">
         <v>294</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="21" t="s">
         <v>302</v>
       </c>
-      <c r="G5" s="23" t="b">
+      <c r="G5" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H5" s="22" t="s">
+      <c r="H5" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="K5" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="21" t="s">
         <v>304</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="21" t="s">
         <v>305</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="21" t="s">
         <v>299</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="21" t="s">
         <v>302</v>
       </c>
-      <c r="G6" s="23" t="b">
+      <c r="G6" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H6" s="22" t="s">
+      <c r="H6" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="I6" s="22" t="n">
+      <c r="I6" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J6" s="22" t="n">
+      <c r="J6" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K6" s="22" t="n">
+      <c r="K6" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="21" t="s">
         <v>169</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="21" t="s">
         <v>306</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="21" t="s">
         <v>307</v>
       </c>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" s="21" t="s">
         <v>296</v>
       </c>
-      <c r="G7" s="23" t="b">
+      <c r="G7" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H7" s="22" t="s">
+      <c r="H7" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="I7" s="22" t="n">
+      <c r="I7" s="21" t="n">
         <v>0.8</v>
       </c>
-      <c r="J7" s="22" t="n">
+      <c r="J7" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="K7" s="22" t="n">
+      <c r="K7" s="21" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="21" t="s">
         <v>308</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="21" t="s">
         <v>309</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="21" t="s">
         <v>307</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="F8" s="21" t="s">
         <v>302</v>
       </c>
-      <c r="G8" s="23" t="b">
+      <c r="G8" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H8" s="22" t="s">
+      <c r="H8" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="I8" s="22" t="n">
+      <c r="I8" s="21" t="n">
         <v>0.8</v>
       </c>
-      <c r="J8" s="22" t="n">
+      <c r="J8" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="K8" s="22" t="n">
+      <c r="K8" s="21" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Use robot localization package to perform global localization
</commit_message>
<xml_diff>
--- a/config/Configuration-Test.xlsx
+++ b/config/Configuration-Test.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -154,7 +154,7 @@
     <t xml:space="preserve">Operational Conditions O1</t>
   </si>
   <si>
-    <t xml:space="preserve">(lat=35.9865559, lon=-5.8930106, alt=8.54)</t>
+    <t xml:space="preserve">(lat=35.9865559, lon=-5.8930106, alt=0.0)</t>
   </si>
   <si>
     <t xml:space="preserve">(Vx=3.0, Vy=1.5, Vz=0.0)</t>

</xml_diff>

<commit_message>
Achieve correct global positioning
</commit_message>
<xml_diff>
--- a/config/Configuration-Test.xlsx
+++ b/config/Configuration-Test.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="321">
   <si>
     <t xml:space="preserve">GENERAL CONFIGURATION</t>
   </si>
@@ -275,6 +275,9 @@
   </si>
   <si>
     <t xml:space="preserve">TRACKING01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(X=10.0, Y=-2.5, Z=0.0)</t>
   </si>
   <si>
     <t xml:space="preserve">AGENT02</t>
@@ -995,10 +998,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -1161,7 +1165,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1247,6 +1251,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1730,7 +1738,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="21" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="21" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.44"/>
@@ -2298,7 +2306,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD16"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="2" width="29.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="40.25"/>
@@ -2313,7 +2321,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -2334,62 +2342,62 @@
         <v>2</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>316</v>
-      </c>
-      <c r="C3" s="21" t="b">
+        <v>317</v>
+      </c>
+      <c r="C3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>317</v>
-      </c>
-      <c r="E3" s="21" t="b">
+        <v>318</v>
+      </c>
+      <c r="E3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>318</v>
-      </c>
-      <c r="G3" s="21" t="b">
+        <v>319</v>
+      </c>
+      <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="I3" s="21" t="n">
         <v>0.4</v>
@@ -2437,7 +2445,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="33.54"/>
@@ -2528,7 +2536,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:BM1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="38.38"/>
@@ -2980,7 +2988,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD20"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -3107,7 +3115,7 @@
         <v>77</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G4" s="18" t="s">
         <v>78</v>
@@ -3124,16 +3132,16 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C5" s="18" t="s">
         <v>27</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E5" s="18" t="s">
         <v>77</v>
@@ -3158,16 +3166,16 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C6" s="18" t="s">
         <v>31</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E6" s="18" t="s">
         <v>77</v>
@@ -3190,22 +3198,22 @@
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C7" s="18" t="s">
         <v>31</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E7" s="18" t="s">
         <v>77</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G7" s="18" t="s">
         <v>78</v>
@@ -3222,22 +3230,22 @@
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C8" s="18" t="s">
         <v>31</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E8" s="18" t="s">
         <v>77</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G8" s="18" t="s">
         <v>78</v>
@@ -3254,16 +3262,16 @@
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>34</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E9" s="18" t="s">
         <v>77</v>
@@ -3286,22 +3294,22 @@
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C10" s="18" t="s">
         <v>34</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E10" s="18" t="s">
         <v>77</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G10" s="18" t="s">
         <v>78</v>
@@ -3318,22 +3326,22 @@
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C11" s="18" t="s">
         <v>34</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E11" s="18" t="s">
         <v>77</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G11" s="18" t="s">
         <v>78</v>
@@ -3350,16 +3358,16 @@
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C12" s="18" t="s">
         <v>37</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E12" s="18" t="s">
         <v>77</v>
@@ -3382,22 +3390,22 @@
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C13" s="18" t="s">
         <v>37</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E13" s="18" t="s">
         <v>77</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G13" s="18" t="s">
         <v>78</v>
@@ -3414,22 +3422,22 @@
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C14" s="18" t="s">
         <v>37</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E14" s="18" t="s">
         <v>77</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G14" s="18" t="s">
         <v>78</v>
@@ -3473,7 +3481,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD24"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -3506,16 +3514,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H2" s="12"/>
       <c r="I2" s="12"/>
@@ -3534,10 +3542,10 @@
         <v>76</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D3" s="18" t="n">
         <v>0.2</v>
@@ -3559,10 +3567,10 @@
         <v>81</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D4" s="18" t="n">
         <v>0.2</v>
@@ -3581,13 +3589,13 @@
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D5" s="18" t="n">
         <v>0.2</v>
@@ -3611,13 +3619,13 @@
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D6" s="18" t="n">
         <v>0.2</v>
@@ -3636,13 +3644,13 @@
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>0.2</v>
@@ -3661,13 +3669,13 @@
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>0.2</v>
@@ -3686,13 +3694,13 @@
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D9" s="18" t="n">
         <v>0.2</v>
@@ -3711,13 +3719,13 @@
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D10" s="18" t="n">
         <v>0.2</v>
@@ -3736,13 +3744,13 @@
     </row>
     <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D11" s="18" t="n">
         <v>0.2</v>
@@ -3761,13 +3769,13 @@
     </row>
     <row r="12" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D12" s="18" t="n">
         <v>0.2</v>
@@ -3786,13 +3794,13 @@
     </row>
     <row r="13" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D13" s="18" t="n">
         <v>0.2</v>
@@ -3811,13 +3819,13 @@
     </row>
     <row r="14" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D14" s="18" t="n">
         <v>0.2</v>
@@ -3867,7 +3875,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD32"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.28"/>
@@ -3904,31 +3912,31 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H2" s="17" t="s">
         <v>70</v>
       </c>
       <c r="I2" s="17" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="K2" s="17" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="M2" s="12"/>
       <c r="N2" s="12"/>
@@ -3936,28 +3944,28 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I3" s="18" t="n">
         <v>3</v>
@@ -3972,28 +3980,28 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I4" s="18" t="n">
         <v>8</v>
@@ -4008,28 +4016,28 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I5" s="18" t="n">
         <v>8</v>
@@ -4044,28 +4052,28 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I6" s="18" t="n">
         <v>8</v>
@@ -4080,28 +4088,28 @@
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I7" s="18" t="n">
         <v>8</v>
@@ -4116,28 +4124,28 @@
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I8" s="18" t="n">
         <v>3</v>
@@ -4153,28 +4161,28 @@
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="B9" s="18" t="s">
-        <v>171</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>117</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>169</v>
-      </c>
       <c r="E9" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I9" s="18" t="n">
         <v>3</v>
@@ -4189,28 +4197,28 @@
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I10" s="18" t="n">
         <v>8</v>
@@ -4225,28 +4233,28 @@
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I11" s="18" t="n">
         <v>8</v>
@@ -4261,28 +4269,28 @@
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I12" s="18" t="n">
         <v>3</v>
@@ -4297,28 +4305,28 @@
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I13" s="18" t="n">
         <v>8</v>
@@ -4333,28 +4341,28 @@
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I14" s="18" t="n">
         <v>8</v>
@@ -4369,28 +4377,28 @@
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I15" s="18" t="n">
         <v>3</v>
@@ -4405,28 +4413,28 @@
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H16" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I16" s="18" t="n">
         <v>8</v>
@@ -4441,28 +4449,28 @@
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H17" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I17" s="18" t="n">
         <v>8</v>
@@ -4477,28 +4485,28 @@
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I18" s="18" t="n">
         <v>3</v>
@@ -4513,28 +4521,28 @@
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G19" s="18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H19" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I19" s="18" t="n">
         <v>8</v>
@@ -4549,28 +4557,28 @@
     </row>
     <row r="20" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G20" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H20" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I20" s="18" t="n">
         <v>8</v>
@@ -4585,28 +4593,28 @@
     </row>
     <row r="21" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H21" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I21" s="18" t="n">
         <v>3</v>
@@ -4622,28 +4630,28 @@
     </row>
     <row r="22" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G22" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H22" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I22" s="18" t="n">
         <v>3</v>
@@ -4659,28 +4667,28 @@
     </row>
     <row r="23" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G23" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H23" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I23" s="18" t="n">
         <v>3</v>
@@ -4696,28 +4704,28 @@
     </row>
     <row r="24" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H24" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I24" s="18" t="n">
         <v>3</v>
@@ -4732,28 +4740,28 @@
     </row>
     <row r="25" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G25" s="18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H25" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I25" s="18" t="n">
         <v>8</v>
@@ -4768,28 +4776,28 @@
     </row>
     <row r="26" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G26" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H26" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I26" s="18" t="n">
         <v>8</v>
@@ -4804,28 +4812,28 @@
     </row>
     <row r="27" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G27" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H27" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I27" s="18" t="n">
         <v>3</v>
@@ -4840,28 +4848,28 @@
     </row>
     <row r="28" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G28" s="18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H28" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I28" s="18" t="n">
         <v>8</v>
@@ -4876,28 +4884,28 @@
     </row>
     <row r="29" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="18" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F29" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G29" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H29" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I29" s="18" t="n">
         <v>8</v>
@@ -4912,28 +4920,28 @@
     </row>
     <row r="30" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G30" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H30" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I30" s="18" t="n">
         <v>3</v>
@@ -4948,28 +4956,28 @@
     </row>
     <row r="31" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="18" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D31" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G31" s="18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H31" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I31" s="18" t="n">
         <v>8</v>
@@ -4984,28 +4992,28 @@
     </row>
     <row r="32" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F32" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G32" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H32" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I32" s="18" t="n">
         <v>8</v>
@@ -5041,7 +5049,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD20"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.28"/>
@@ -5072,19 +5080,19 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="XEV2" s="3"/>
       <c r="XEW2" s="3"/>
@@ -5098,16 +5106,16 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E3" s="18" t="n">
         <v>0.167</v>
@@ -5121,16 +5129,16 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="18" t="s">
         <v>225</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>226</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>224</v>
       </c>
       <c r="E4" s="18" t="n">
         <v>0.167</v>
@@ -5144,16 +5152,16 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E5" s="18" t="n">
         <v>0.167</v>
@@ -5167,16 +5175,16 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E6" s="18" t="n">
         <v>0.167</v>
@@ -5190,16 +5198,16 @@
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E7" s="18" t="n">
         <v>0.167</v>
@@ -5213,16 +5221,16 @@
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E8" s="18" t="n">
         <v>0.167</v>
@@ -5236,16 +5244,16 @@
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E9" s="18" t="n">
         <v>0.167</v>
@@ -5259,16 +5267,16 @@
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E10" s="18" t="n">
         <v>0.167</v>
@@ -5282,16 +5290,16 @@
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E11" s="18" t="n">
         <v>0.167</v>
@@ -5305,16 +5313,16 @@
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E12" s="18" t="n">
         <v>0.167</v>
@@ -5328,16 +5336,16 @@
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>0.167</v>
@@ -5351,16 +5359,16 @@
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E14" s="18" t="n">
         <v>0.167</v>
@@ -5374,16 +5382,16 @@
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E15" s="18" t="n">
         <v>0.167</v>
@@ -5397,16 +5405,16 @@
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E16" s="18" t="n">
         <v>0.167</v>
@@ -5420,16 +5428,16 @@
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E17" s="18" t="n">
         <v>0.167</v>
@@ -5443,16 +5451,16 @@
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E18" s="18" t="n">
         <v>0.167</v>
@@ -5466,16 +5474,16 @@
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E19" s="18" t="n">
         <v>0.167</v>
@@ -5489,16 +5497,16 @@
     </row>
     <row r="20" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E20" s="18" t="n">
         <v>0.167</v>
@@ -5533,7 +5541,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:R1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="34.63"/>
@@ -5552,7 +5560,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -5583,49 +5591,49 @@
         <v>46</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="L2" s="20" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="M2" s="20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="N2" s="20" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="O2" s="20" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="P2" s="20" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q2" s="20" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="R2" s="20" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5636,7 +5644,7 @@
         <v>40</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D3" s="21" t="n">
         <v>8</v>
@@ -5644,33 +5652,33 @@
       <c r="E3" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="21" t="b">
+      <c r="F3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>276</v>
-      </c>
-      <c r="H3" s="21" t="b">
+        <v>277</v>
+      </c>
+      <c r="H3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I3" s="21" t="s">
-        <v>277</v>
-      </c>
-      <c r="J3" s="21" t="b">
+        <v>278</v>
+      </c>
+      <c r="J3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K3" s="21" t="s">
-        <v>278</v>
-      </c>
-      <c r="L3" s="21" t="b">
+        <v>279</v>
+      </c>
+      <c r="L3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="N3" s="21" t="n">
         <v>6.5</v>
@@ -5690,13 +5698,13 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B4" s="21" t="s">
         <v>44</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D4" s="21" t="n">
         <v>8</v>
@@ -5704,33 +5712,33 @@
       <c r="E4" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F4" s="21" t="b">
+      <c r="F4" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>281</v>
-      </c>
-      <c r="H4" s="21" t="b">
+        <v>282</v>
+      </c>
+      <c r="H4" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I4" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="J4" s="21" t="b">
+        <v>283</v>
+      </c>
+      <c r="J4" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K4" s="21" t="s">
-        <v>283</v>
-      </c>
-      <c r="L4" s="21" t="b">
+        <v>284</v>
+      </c>
+      <c r="L4" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="M4" s="21" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="N4" s="21" t="n">
         <v>6.5</v>
@@ -5787,7 +5795,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD21"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="63.93"/>
@@ -5804,7 +5812,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -5828,28 +5836,28 @@
         <v>46</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="XFB2" s="3"/>
       <c r="XFC2" s="3"/>
@@ -5857,29 +5865,29 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>296</v>
-      </c>
-      <c r="G3" s="21" t="b">
+        <v>297</v>
+      </c>
+      <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="I3" s="21" t="n">
         <v>0.5</v>
@@ -5893,29 +5901,29 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>296</v>
-      </c>
-      <c r="G4" s="21" t="b">
+        <v>297</v>
+      </c>
+      <c r="G4" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="I4" s="21" t="n">
         <v>0.5</v>
@@ -5929,29 +5937,29 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>302</v>
-      </c>
-      <c r="G5" s="21" t="b">
+        <v>303</v>
+      </c>
+      <c r="G5" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I5" s="21" t="n">
         <v>0.5</v>
@@ -5965,29 +5973,29 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>302</v>
-      </c>
-      <c r="G6" s="21" t="b">
+        <v>303</v>
+      </c>
+      <c r="G6" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H6" s="21" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I6" s="21" t="n">
         <v>0.5</v>
@@ -6001,29 +6009,29 @@
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>296</v>
-      </c>
-      <c r="G7" s="21" t="b">
+        <v>297</v>
+      </c>
+      <c r="G7" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H7" s="21" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="I7" s="21" t="n">
         <v>0.8</v>
@@ -6037,29 +6045,29 @@
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
+        <v>309</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>310</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>294</v>
+      </c>
+      <c r="D8" s="21" t="s">
         <v>308</v>
       </c>
-      <c r="B8" s="21" t="s">
-        <v>309</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>293</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>307</v>
-      </c>
       <c r="E8" s="21" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>302</v>
-      </c>
-      <c r="G8" s="21" t="b">
+        <v>303</v>
+      </c>
+      <c r="G8" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H8" s="21" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I8" s="21" t="n">
         <v>0.8</v>

</xml_diff>

<commit_message>
Add stream configuration for AirSim
</commit_message>
<xml_diff>
--- a/config/Configuration-Test.xlsx
+++ b/config/Configuration-Test.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -463,7 +463,7 @@
     <t xml:space="preserve">RefFocal [mm]</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTICAMERA0</t>
+    <t xml:space="preserve">MULTICAMERA00</t>
   </si>
   <si>
     <t xml:space="preserve">Central Head Multi-Camera (Single)</t>
@@ -484,7 +484,7 @@
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=90.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTICAMERA1</t>
+    <t xml:space="preserve">MULTICAMERA01</t>
   </si>
   <si>
     <t xml:space="preserve">Tracking Head 1 Multi-Camera (Single)</t>
@@ -502,7 +502,7 @@
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=0.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTICAMERA2</t>
+    <t xml:space="preserve">MULTICAMERA02</t>
   </si>
   <si>
     <t xml:space="preserve">Tracking Head 2 Multi-Camera (Single)</t>
@@ -511,7 +511,7 @@
     <t xml:space="preserve">(X=0.0, Y=0.3, Z=-0.15)</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTICAMERA3</t>
+    <t xml:space="preserve">MULTICAMERA03</t>
   </si>
   <si>
     <t xml:space="preserve">Tracking Head 3 Multi-Camera (Single)</t>
@@ -523,7 +523,7 @@
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=180.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTICAMERA4</t>
+    <t xml:space="preserve">MULTICAMERA04</t>
   </si>
   <si>
     <t xml:space="preserve">Tracking Head 4 Multi-Camera (Single)</t>
@@ -535,7 +535,7 @@
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=270.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTICAMERA5</t>
+    <t xml:space="preserve">MULTICAMERA05</t>
   </si>
   <si>
     <t xml:space="preserve">Central Head Multi-Window (Single)</t>
@@ -544,25 +544,25 @@
     <t xml:space="preserve">CAM04</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTICAMERA6</t>
+    <t xml:space="preserve">MULTICAMERA06</t>
   </si>
   <si>
     <t xml:space="preserve">Central Head Multi-Hybrid (Single)</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTICAMERA7</t>
+    <t xml:space="preserve">MULTICAMERA07</t>
   </si>
   <si>
     <t xml:space="preserve">Tracking Head 1 Multi-Hybrid (Single)</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTICAMERA8</t>
+    <t xml:space="preserve">MULTICAMERA08</t>
   </si>
   <si>
     <t xml:space="preserve">Tracking Head 2 Multi-Hybrid (Single)</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTICAMERA9</t>
+    <t xml:space="preserve">MULTICAMERA09</t>
   </si>
   <si>
     <t xml:space="preserve">Central Head Multi-Camera 1 (Multi)</t>
@@ -998,11 +998,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0"/>
-    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -1165,7 +1164,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1251,10 +1250,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1738,7 +1733,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="21" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="21" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.44"/>
@@ -2306,7 +2301,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD16"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="2" width="29.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="40.25"/>
@@ -2378,21 +2373,21 @@
       <c r="B3" s="21" t="s">
         <v>317</v>
       </c>
-      <c r="C3" s="22" t="b">
+      <c r="C3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D3" s="21" t="s">
         <v>318</v>
       </c>
-      <c r="E3" s="22" t="b">
+      <c r="E3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="F3" s="21" t="s">
         <v>319</v>
       </c>
-      <c r="G3" s="22" t="b">
+      <c r="G3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2445,7 +2440,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="33.54"/>
@@ -2536,7 +2531,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:BM1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="38.38"/>
@@ -2988,7 +2983,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD20"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -3481,7 +3476,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD24"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -3875,7 +3870,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD32"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.28"/>
@@ -5049,7 +5044,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD20"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.28"/>
@@ -5541,7 +5536,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:R1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="34.63"/>
@@ -5652,28 +5647,28 @@
       <c r="E3" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="22" t="b">
+      <c r="F3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="G3" s="21" t="s">
         <v>277</v>
       </c>
-      <c r="H3" s="22" t="b">
+      <c r="H3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I3" s="21" t="s">
         <v>278</v>
       </c>
-      <c r="J3" s="22" t="b">
+      <c r="J3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K3" s="21" t="s">
         <v>279</v>
       </c>
-      <c r="L3" s="22" t="b">
+      <c r="L3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5712,28 +5707,28 @@
       <c r="E4" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F4" s="22" t="b">
+      <c r="F4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="G4" s="21" t="s">
         <v>282</v>
       </c>
-      <c r="H4" s="22" t="b">
+      <c r="H4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I4" s="21" t="s">
         <v>283</v>
       </c>
-      <c r="J4" s="22" t="b">
+      <c r="J4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K4" s="21" t="s">
         <v>284</v>
       </c>
-      <c r="L4" s="22" t="b">
+      <c r="L4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5795,7 +5790,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD21"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="63.93"/>
@@ -5882,7 +5877,7 @@
       <c r="F3" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="G3" s="22" t="b">
+      <c r="G3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5918,7 +5913,7 @@
       <c r="F4" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="G4" s="22" t="b">
+      <c r="G4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5954,7 +5949,7 @@
       <c r="F5" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="G5" s="22" t="b">
+      <c r="G5" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -5990,7 +5985,7 @@
       <c r="F6" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="G6" s="22" t="b">
+      <c r="G6" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -6026,7 +6021,7 @@
       <c r="F7" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="G7" s="22" t="b">
+      <c r="G7" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -6062,7 +6057,7 @@
       <c r="F8" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="G8" s="22" t="b">
+      <c r="G8" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Create GUI setpoints signal for operator interface
</commit_message>
<xml_diff>
--- a/config/Configuration-Test.xlsx
+++ b/config/Configuration-Test.xlsx
@@ -1102,18 +1102,18 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="2" tint="-0.75"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1240,7 +1240,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1252,7 +1252,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1260,7 +1260,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1923,7 +1923,7 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="8" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="9" t="s">
@@ -2003,7 +2003,7 @@
       <c r="BD4" s="12"/>
     </row>
     <row r="5" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="9" t="s">
         <v>25</v>
       </c>
@@ -2081,7 +2081,7 @@
       <c r="BD5" s="12"/>
     </row>
     <row r="6" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="9" t="s">
         <v>28</v>
       </c>
@@ -2159,7 +2159,7 @@
       <c r="BD6" s="12"/>
     </row>
     <row r="7" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8"/>
+      <c r="A7" s="13"/>
       <c r="B7" s="9" t="s">
         <v>32</v>
       </c>
@@ -2237,7 +2237,7 @@
       <c r="BD7" s="12"/>
     </row>
     <row r="8" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8"/>
+      <c r="A8" s="13"/>
       <c r="B8" s="9" t="s">
         <v>35</v>
       </c>

</xml_diff>